<commit_message>
Remove Name from import template fields
</commit_message>
<xml_diff>
--- a/public/templates/realdeal-contact-import-template.xlsx
+++ b/public/templates/realdeal-contact-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" r:id="R6b98b20a15154452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R0cff339440414148"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="R40558481ad5d494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" r:id="R48c721d8a00d45d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R5558a6676fb1422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" r:id="Ra8a5bd7ed3094d74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -273,83 +273,81 @@
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Name</x:v>
+        <x:v>First Name</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>First Name</x:v>
+        <x:v>Last Name</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Last Name</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Email</x:v>
+        <x:v>Phone</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Phone</x:v>
+        <x:v>Company</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Company</x:v>
+        <x:v>Role</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>Role</x:v>
+        <x:v>Pod</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>Pod</x:v>
+        <x:v>Sub-pod</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>Sub-pod</x:v>
+        <x:v>Contact Frequency</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>Contact Frequency</x:v>
+        <x:v>Last Contacted</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>Last Contacted</x:v>
+        <x:v>Next Follow Up Date</x:v>
       </x:c>
       <x:c r="L1" s="3" t="str">
-        <x:v>Next Follow Up Date</x:v>
+        <x:v>Next Action</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>Next Action</x:v>
+        <x:v>Relationship Context</x:v>
       </x:c>
       <x:c r="N1" s="3" t="str">
-        <x:v>Relationship Context</x:v>
+        <x:v>Intel Notes</x:v>
       </x:c>
       <x:c r="O1" s="3" t="str">
-        <x:v>Intel Notes</x:v>
+        <x:v>Relationship Owner</x:v>
       </x:c>
       <x:c r="P1" s="3" t="str">
-        <x:v>Relationship Owner</x:v>
+        <x:v>Introduced By</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="str">
-        <x:v>Introduced By</x:v>
+        <x:v>LinkedIn</x:v>
       </x:c>
       <x:c r="R1" s="3" t="str">
-        <x:v>LinkedIn</x:v>
+        <x:v>Website</x:v>
       </x:c>
       <x:c r="S1" s="3" t="str">
-        <x:v>Website</x:v>
+        <x:v>Location</x:v>
       </x:c>
       <x:c r="T1" s="3" t="str">
-        <x:v>Location</x:v>
+        <x:v>Country</x:v>
       </x:c>
       <x:c r="U1" s="3" t="str">
-        <x:v>Country</x:v>
+        <x:v>Notes</x:v>
       </x:c>
       <x:c r="V1" s="3" t="str">
-        <x:v>Notes</x:v>
+        <x:v>KV Fund Investor</x:v>
       </x:c>
       <x:c r="W1" s="3" t="str">
-        <x:v>KV Fund Investor</x:v>
+        <x:v>SPV Investor</x:v>
       </x:c>
       <x:c r="X1" s="3" t="str">
-        <x:v>SPV Investor</x:v>
+        <x:v>Email 2</x:v>
       </x:c>
       <x:c r="Y1" s="3" t="str">
-        <x:v>Email 2</x:v>
-      </x:c>
-      <x:c r="Z1" s="3" t="str">
         <x:v>Email 3</x:v>
       </x:c>
+      <x:c r="Z1" s="3"/>
       <x:c r="AA1" s="3" t="str">
         <x:v>Birthday</x:v>
       </x:c>
@@ -5392,7 +5390,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
-        <x:v>Fill either Name OR First Name + Last Name. Pod is strongly recommended; if left blank during upload, select a fallback pod in the app.</x:v>
+        <x:v>Fill First Name and Last Name when available. If an imported file only has Name, Real Deal stores that value in First Name. Pod is strongly recommended; if left blank during upload, select a fallback pod in the app.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5491,227 +5489,221 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Name</x:v>
+        <x:v>First Name</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>First Name</x:v>
+        <x:v>Last Name</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Last Name</x:v>
+        <x:v>Email</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Email</x:v>
+        <x:v>Phone</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Phone</x:v>
+        <x:v>Company</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Company</x:v>
+        <x:v>Role</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>Role</x:v>
+        <x:v>Pod</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>Pod</x:v>
+        <x:v>Sub-pod</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>Sub-pod</x:v>
+        <x:v>Contact Frequency</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>Contact Frequency</x:v>
+        <x:v>Last Contacted</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>Last Contacted</x:v>
+        <x:v>Next Follow Up Date</x:v>
       </x:c>
       <x:c r="L1" s="3" t="str">
-        <x:v>Next Follow Up Date</x:v>
+        <x:v>Next Action</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>Next Action</x:v>
+        <x:v>Relationship Context</x:v>
       </x:c>
       <x:c r="N1" s="3" t="str">
-        <x:v>Relationship Context</x:v>
+        <x:v>Intel Notes</x:v>
       </x:c>
       <x:c r="O1" s="3" t="str">
-        <x:v>Intel Notes</x:v>
+        <x:v>Relationship Owner</x:v>
       </x:c>
       <x:c r="P1" s="3" t="str">
-        <x:v>Relationship Owner</x:v>
+        <x:v>Introduced By</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="str">
-        <x:v>Introduced By</x:v>
+        <x:v>LinkedIn</x:v>
       </x:c>
       <x:c r="R1" s="3" t="str">
-        <x:v>LinkedIn</x:v>
+        <x:v>Website</x:v>
       </x:c>
       <x:c r="S1" s="3" t="str">
-        <x:v>Website</x:v>
+        <x:v>Location</x:v>
       </x:c>
       <x:c r="T1" s="3" t="str">
-        <x:v>Location</x:v>
+        <x:v>Country</x:v>
       </x:c>
       <x:c r="U1" s="3" t="str">
-        <x:v>Country</x:v>
+        <x:v>Notes</x:v>
       </x:c>
       <x:c r="V1" s="3" t="str">
-        <x:v>Notes</x:v>
+        <x:v>KV Fund Investor</x:v>
       </x:c>
       <x:c r="W1" s="3" t="str">
-        <x:v>KV Fund Investor</x:v>
+        <x:v>SPV Investor</x:v>
       </x:c>
       <x:c r="X1" s="3" t="str">
-        <x:v>SPV Investor</x:v>
+        <x:v>Email 2</x:v>
       </x:c>
       <x:c r="Y1" s="3" t="str">
-        <x:v>Email 2</x:v>
-      </x:c>
-      <x:c r="Z1" s="3" t="str">
         <x:v>Email 3</x:v>
       </x:c>
+      <x:c r="Z1" s="3"/>
       <x:c r="AA1" s="3" t="str">
         <x:v>Birthday</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Emily Tran</x:v>
+        <x:v>Emily</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Emily</x:v>
+        <x:v>Tran</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Tran</x:v>
+        <x:v>emily@example.com</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>emily@example.com</x:v>
+        <x:v>+1 555 0100</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>+1 555 0100</x:v>
+        <x:v>Tran Family Office</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>Tran Family Office</x:v>
+        <x:v>CIO</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>CIO</x:v>
+        <x:v>LPs</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>LPs</x:v>
+        <x:v>Family Offices</x:v>
       </x:c>
       <x:c r="I2" t="str">
-        <x:v>Family Offices</x:v>
+        <x:v>Monthly</x:v>
       </x:c>
       <x:c r="J2" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>2026-05-01</x:v>
       </x:c>
       <x:c r="K2" s="4" t="str">
-        <x:v>2026-05-01</x:v>
+        <x:v>2026-06-01</x:v>
       </x:c>
       <x:c r="L2" s="4" t="str">
-        <x:v>2026-06-01</x:v>
+        <x:v>Send Q2 LP update</x:v>
       </x:c>
       <x:c r="M2" t="str">
-        <x:v>Send Q2 LP update</x:v>
+        <x:v>Committed to Fund II and is warm for Fund III.</x:v>
       </x:c>
       <x:c r="N2" t="str">
-        <x:v>Committed to Fund II and is warm for Fund III.</x:v>
+        <x:v>Prefers concise fund updates and direct asks.</x:v>
       </x:c>
       <x:c r="O2" t="str">
-        <x:v>Prefers concise fund updates and direct asks.</x:v>
+        <x:v>Moj</x:v>
       </x:c>
       <x:c r="P2" t="str">
-        <x:v>Moj</x:v>
+        <x:v>Sarah Chen</x:v>
       </x:c>
       <x:c r="Q2" t="str">
-        <x:v>Sarah Chen</x:v>
+        <x:v>https://linkedin.com/in/example</x:v>
       </x:c>
       <x:c r="R2" t="str">
-        <x:v>https://linkedin.com/in/example</x:v>
+        <x:v>https://example.com</x:v>
       </x:c>
       <x:c r="S2" t="str">
-        <x:v>https://example.com</x:v>
+        <x:v>San Francisco</x:v>
       </x:c>
       <x:c r="T2" t="str">
-        <x:v>San Francisco</x:v>
+        <x:v>United States</x:v>
       </x:c>
       <x:c r="U2" t="str">
-        <x:v>United States</x:v>
+        <x:v>Met at investor dinner.</x:v>
       </x:c>
       <x:c r="V2" t="str">
-        <x:v>Met at investor dinner.</x:v>
+        <x:v>Fund II</x:v>
       </x:c>
       <x:c r="W2" t="str">
-        <x:v>Fund II</x:v>
-      </x:c>
-      <x:c r="X2" t="str">
         <x:v>SPV-Glossier</x:v>
       </x:c>
+      <x:c r="X2" t="str"/>
       <x:c r="Y2" t="str"/>
-      <x:c r="Z2" t="str"/>
+      <x:c r="Z2"/>
       <x:c r="AA2" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Robert Okafor</x:v>
+        <x:v>Robert</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Robert</x:v>
+        <x:v>Okafor</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Okafor</x:v>
+        <x:v>robert@example.com</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>robert@example.com</x:v>
+        <x:v>+1 555 0101</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>+1 555 0101</x:v>
+        <x:v>Okafor Capital</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>Okafor Capital</x:v>
+        <x:v>Founder</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>Founder</x:v>
+        <x:v>LPs</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>LPs</x:v>
+        <x:v>Angels</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>Angels</x:v>
+        <x:v>Quarterly</x:v>
       </x:c>
       <x:c r="J3" t="str">
-        <x:v>Quarterly</x:v>
-      </x:c>
-      <x:c r="K3" s="4" t="str">
         <x:v>2026-04-15</x:v>
       </x:c>
-      <x:c r="L3" s="4" t="str"/>
+      <x:c r="K3" s="4" t="str"/>
+      <x:c r="L3" s="4" t="str">
+        <x:v>Quarterly check-in</x:v>
+      </x:c>
       <x:c r="M3" t="str">
-        <x:v>Quarterly check-in</x:v>
+        <x:v>Warm but slow mover.</x:v>
       </x:c>
       <x:c r="N3" t="str">
-        <x:v>Warm but slow mover.</x:v>
+        <x:v>Needs context before committing.</x:v>
       </x:c>
       <x:c r="O3" t="str">
-        <x:v>Needs context before committing.</x:v>
-      </x:c>
-      <x:c r="P3" t="str">
         <x:v>Briell</x:v>
       </x:c>
+      <x:c r="P3" t="str"/>
       <x:c r="Q3" t="str"/>
       <x:c r="R3" t="str"/>
-      <x:c r="S3" t="str"/>
+      <x:c r="S3" t="str">
+        <x:v>Chicago</x:v>
+      </x:c>
       <x:c r="T3" t="str">
-        <x:v>Chicago</x:v>
-      </x:c>
-      <x:c r="U3" t="str">
         <x:v>United States</x:v>
       </x:c>
-      <x:c r="V3" t="str"/>
-      <x:c r="W3" t="str">
+      <x:c r="U3" t="str"/>
+      <x:c r="V3" t="str">
         <x:v>Fund I</x:v>
       </x:c>
+      <x:c r="W3" t="str"/>
       <x:c r="X3" t="str"/>
       <x:c r="Y3" t="str"/>
-      <x:c r="Z3" t="str"/>
+      <x:c r="Z3"/>
       <x:c r="AA3" t="str"/>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add required LP contact fields
</commit_message>
<xml_diff>
--- a/public/templates/realdeal-contact-import-template.xlsx
+++ b/public/templates/realdeal-contact-import-template.xlsx
@@ -329,7 +329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP1"/>
+  <dimension ref="A1:BS1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -400,6 +400,9 @@
     <col width="20" customWidth="1" min="66" max="66"/>
     <col width="15" customWidth="1" min="67" max="67"/>
     <col width="14" customWidth="1" min="68" max="68"/>
+    <col width="18" customWidth="1" min="69" max="69"/>
+    <col width="22" customWidth="1" min="70" max="70"/>
+    <col width="34" customWidth="1" min="71" max="71"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1">
@@ -610,7 +613,7 @@
       </c>
       <c r="AP1" s="13" t="inlineStr">
         <is>
-          <t>Fundraise Status</t>
+          <t>KV Status</t>
         </is>
       </c>
       <c r="AQ1" s="13" t="inlineStr">
@@ -743,9 +746,24 @@
           <t>Comments</t>
         </is>
       </c>
+      <c r="BQ1" s="13" t="inlineStr">
+        <is>
+          <t>Contact Source</t>
+        </is>
+      </c>
+      <c r="BR1" s="13" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="BS1" s="13" t="inlineStr">
+        <is>
+          <t>Company Overview</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BP1"/>
+  <autoFilter ref="A1:BS1"/>
   <dataValidations count="2">
     <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"MAPS,LPs,Companies,Talent &amp; Influencers,Services for Founders,Family &amp; Friends"</formula1>
@@ -764,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1489,7 +1507,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Fundraise Status</t>
+          <t>KV Status</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1942,6 +1960,57 @@
       <c r="C69" s="14" t="inlineStr">
         <is>
           <t>Optional approved import field. Unknown spreadsheet columns are preserved in Notes, not new schema fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Contact Source</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>contacts.custom_fields.contactSource</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>Controlled values: Business Card, WhatsApp, or By Association.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>contacts.custom_fields.companyLinkedIn</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>Company public LinkedIn URL when available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Company Overview</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>contacts.custom_fields.companyOverview</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>Public company context stored with the contact.</t>
         </is>
       </c>
     </row>
@@ -1956,7 +2025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP2"/>
+  <dimension ref="A1:BS2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2027,6 +2096,9 @@
     <col width="20" customWidth="1" min="66" max="66"/>
     <col width="15" customWidth="1" min="67" max="67"/>
     <col width="14" customWidth="1" min="68" max="68"/>
+    <col width="18" customWidth="1" min="69" max="69"/>
+    <col width="22" customWidth="1" min="70" max="70"/>
+    <col width="34" customWidth="1" min="71" max="71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2237,7 +2309,7 @@
       </c>
       <c r="AP1" s="13" t="inlineStr">
         <is>
-          <t>Fundraise Status</t>
+          <t>KV Status</t>
         </is>
       </c>
       <c r="AQ1" s="13" t="inlineStr">
@@ -2368,6 +2440,21 @@
       <c r="BP1" s="13" t="inlineStr">
         <is>
           <t>Comments</t>
+        </is>
+      </c>
+      <c r="BQ1" s="12" t="inlineStr">
+        <is>
+          <t>Contact Source</t>
+        </is>
+      </c>
+      <c r="BR1" s="12" t="inlineStr">
+        <is>
+          <t>Company LinkedIn</t>
+        </is>
+      </c>
+      <c r="BS1" s="12" t="inlineStr">
+        <is>
+          <t>Company Overview</t>
         </is>
       </c>
     </row>
@@ -2544,9 +2631,24 @@
       <c r="BN2" t="inlineStr"/>
       <c r="BO2" t="inlineStr"/>
       <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" s="0" t="inlineStr">
+        <is>
+          <t>Business Card</t>
+        </is>
+      </c>
+      <c r="BR2" s="0" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/moonpay/</t>
+        </is>
+      </c>
+      <c r="BS2" s="0" t="inlineStr">
+        <is>
+          <t>MoonPay is a global payments infrastructure company.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BP2"/>
+  <autoFilter ref="A1:BS2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add campaign import mapping
</commit_message>
<xml_diff>
--- a/public/templates/realdeal-contact-import-template.xlsx
+++ b/public/templates/realdeal-contact-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" r:id="Rff0fd5b3d8844b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="2" r:id="Re8a8b4e4104a4151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Options" sheetId="3" r:id="R0614c273f5354e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" r:id="R2c5a757459064d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="2" r:id="Rb76c05515ad74608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Options" sheetId="3" r:id="R39f957ab3d864598"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -106,8 +106,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTemplate" displayName="ContactsTemplate" ref="A1:AD51" headerRowCount="1">
-  <x:tableColumns count="30">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTemplate" displayName="ContactsTemplate" ref="A1:AO51" headerRowCount="1">
+  <x:tableColumns count="41">
     <x:tableColumn id="1" name="Name"/>
     <x:tableColumn id="2" name="Company"/>
     <x:tableColumn id="3" name="Job Title"/>
@@ -136,16 +136,27 @@
     <x:tableColumn id="26" name="Notes"/>
     <x:tableColumn id="27" name="Pods"/>
     <x:tableColumn id="28" name="Sub-pods"/>
-    <x:tableColumn id="29" name="Campaign"/>
-    <x:tableColumn id="30" name="Companies"/>
+    <x:tableColumn id="29" name="Campaign 1"/>
+    <x:tableColumn id="30" name="Campaign 1 Status"/>
+    <x:tableColumn id="31" name="Campaign 1 Target Commitment"/>
+    <x:tableColumn id="32" name="Campaign 2"/>
+    <x:tableColumn id="33" name="Campaign 2 Status"/>
+    <x:tableColumn id="34" name="Campaign 2 Target Commitment"/>
+    <x:tableColumn id="35" name="Campaign 3"/>
+    <x:tableColumn id="36" name="Campaign 3 Status"/>
+    <x:tableColumn id="37" name="Campaign 3 Target Commitment"/>
+    <x:tableColumn id="38" name="Campaign 4"/>
+    <x:tableColumn id="39" name="Campaign 4 Status"/>
+    <x:tableColumn id="40" name="Campaign 4 Target Commitment"/>
+    <x:tableColumn id="41" name="Companies"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CompaniesTemplate" displayName="CompaniesTemplate" ref="A1:R51" headerRowCount="1">
-  <x:tableColumns count="18">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CompaniesTemplate" displayName="CompaniesTemplate" ref="A1:AC51" headerRowCount="1">
+  <x:tableColumns count="29">
     <x:tableColumn id="1" name="Company"/>
     <x:tableColumn id="2" name="Contacts"/>
     <x:tableColumn id="3" name="Website"/>
@@ -163,7 +174,18 @@
     <x:tableColumn id="15" name="Global Region"/>
     <x:tableColumn id="16" name="Pods"/>
     <x:tableColumn id="17" name="Sub-pods"/>
-    <x:tableColumn id="18" name="Campaign"/>
+    <x:tableColumn id="18" name="Campaign 1"/>
+    <x:tableColumn id="19" name="Campaign 1 Status"/>
+    <x:tableColumn id="20" name="Campaign 1 Target Commitment"/>
+    <x:tableColumn id="21" name="Campaign 2"/>
+    <x:tableColumn id="22" name="Campaign 2 Status"/>
+    <x:tableColumn id="23" name="Campaign 2 Target Commitment"/>
+    <x:tableColumn id="24" name="Campaign 3"/>
+    <x:tableColumn id="25" name="Campaign 3 Status"/>
+    <x:tableColumn id="26" name="Campaign 3 Target Commitment"/>
+    <x:tableColumn id="27" name="Campaign 4"/>
+    <x:tableColumn id="28" name="Campaign 4 Status"/>
+    <x:tableColumn id="29" name="Campaign 4 Target Commitment"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -348,6 +370,17 @@
     <x:col min="28" max="28" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="18.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -436,9 +469,42 @@
         <x:v>Sub-pods</x:v>
       </x:c>
       <x:c r="AC1" s="4" t="str">
-        <x:v>Campaign</x:v>
+        <x:v>Campaign 1</x:v>
       </x:c>
       <x:c r="AD1" s="4" t="str">
+        <x:v>Campaign 1 Status</x:v>
+      </x:c>
+      <x:c r="AE1" s="4" t="str">
+        <x:v>Campaign 1 Target Commitment</x:v>
+      </x:c>
+      <x:c r="AF1" s="4" t="str">
+        <x:v>Campaign 2</x:v>
+      </x:c>
+      <x:c r="AG1" s="4" t="str">
+        <x:v>Campaign 2 Status</x:v>
+      </x:c>
+      <x:c r="AH1" s="4" t="str">
+        <x:v>Campaign 2 Target Commitment</x:v>
+      </x:c>
+      <x:c r="AI1" s="4" t="str">
+        <x:v>Campaign 3</x:v>
+      </x:c>
+      <x:c r="AJ1" s="4" t="str">
+        <x:v>Campaign 3 Status</x:v>
+      </x:c>
+      <x:c r="AK1" s="4" t="str">
+        <x:v>Campaign 3 Target Commitment</x:v>
+      </x:c>
+      <x:c r="AL1" s="4" t="str">
+        <x:v>Campaign 4</x:v>
+      </x:c>
+      <x:c r="AM1" s="4" t="str">
+        <x:v>Campaign 4 Status</x:v>
+      </x:c>
+      <x:c r="AN1" s="4" t="str">
+        <x:v>Campaign 4 Target Commitment</x:v>
+      </x:c>
+      <x:c r="AO1" s="4" t="str">
         <x:v>Companies</x:v>
       </x:c>
     </x:row>
@@ -524,8 +590,31 @@
       <x:c r="AB2" s="7" t="str">
         <x:v>LP Internal</x:v>
       </x:c>
-      <x:c r="AC2" s="7" t="str"/>
+      <x:c r="AC2" s="7" t="str">
+        <x:v>Kinship Fund Pipeline</x:v>
+      </x:c>
       <x:c r="AD2" s="7" t="str">
+        <x:v>Closed/Won</x:v>
+      </x:c>
+      <x:c r="AE2" s="7" t="str">
+        <x:v>500000</x:v>
+      </x:c>
+      <x:c r="AF2" s="7" t="str">
+        <x:v>Founder Dinner</x:v>
+      </x:c>
+      <x:c r="AG2" s="7" t="str">
+        <x:v>Invited</x:v>
+      </x:c>
+      <x:c r="AH2" s="7" t="str">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="AI2" s="7" t="str"/>
+      <x:c r="AJ2" s="7" t="str"/>
+      <x:c r="AK2" s="7" t="str"/>
+      <x:c r="AL2" s="7" t="str"/>
+      <x:c r="AM2" s="7" t="str"/>
+      <x:c r="AN2" s="7" t="str"/>
+      <x:c r="AO2" s="7" t="str">
         <x:v>Jahez Group; Namara Investments</x:v>
       </x:c>
     </x:row>
@@ -560,6 +649,17 @@
       <x:c r="AB3" s="7" t="str"/>
       <x:c r="AC3" s="7" t="str"/>
       <x:c r="AD3" s="7" t="str"/>
+      <x:c r="AE3" s="7" t="str"/>
+      <x:c r="AF3" s="7" t="str"/>
+      <x:c r="AG3" s="7" t="str"/>
+      <x:c r="AH3" s="7" t="str"/>
+      <x:c r="AI3" s="7" t="str"/>
+      <x:c r="AJ3" s="7" t="str"/>
+      <x:c r="AK3" s="7" t="str"/>
+      <x:c r="AL3" s="7" t="str"/>
+      <x:c r="AM3" s="7" t="str"/>
+      <x:c r="AN3" s="7" t="str"/>
+      <x:c r="AO3" s="7" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str"/>
@@ -592,6 +692,17 @@
       <x:c r="AB4" s="7" t="str"/>
       <x:c r="AC4" s="7" t="str"/>
       <x:c r="AD4" s="7" t="str"/>
+      <x:c r="AE4" s="7" t="str"/>
+      <x:c r="AF4" s="7" t="str"/>
+      <x:c r="AG4" s="7" t="str"/>
+      <x:c r="AH4" s="7" t="str"/>
+      <x:c r="AI4" s="7" t="str"/>
+      <x:c r="AJ4" s="7" t="str"/>
+      <x:c r="AK4" s="7" t="str"/>
+      <x:c r="AL4" s="7" t="str"/>
+      <x:c r="AM4" s="7" t="str"/>
+      <x:c r="AN4" s="7" t="str"/>
+      <x:c r="AO4" s="7" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="7"/>
@@ -624,6 +735,17 @@
       <x:c r="AB5" s="7"/>
       <x:c r="AC5" s="7"/>
       <x:c r="AD5" s="7"/>
+      <x:c r="AE5" s="7"/>
+      <x:c r="AF5" s="7"/>
+      <x:c r="AG5" s="7"/>
+      <x:c r="AH5" s="7"/>
+      <x:c r="AI5" s="7"/>
+      <x:c r="AJ5" s="7"/>
+      <x:c r="AK5" s="7"/>
+      <x:c r="AL5" s="7"/>
+      <x:c r="AM5" s="7"/>
+      <x:c r="AN5" s="7"/>
+      <x:c r="AO5" s="7"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7"/>
@@ -656,6 +778,17 @@
       <x:c r="AB6" s="7"/>
       <x:c r="AC6" s="7"/>
       <x:c r="AD6" s="7"/>
+      <x:c r="AE6" s="7"/>
+      <x:c r="AF6" s="7"/>
+      <x:c r="AG6" s="7"/>
+      <x:c r="AH6" s="7"/>
+      <x:c r="AI6" s="7"/>
+      <x:c r="AJ6" s="7"/>
+      <x:c r="AK6" s="7"/>
+      <x:c r="AL6" s="7"/>
+      <x:c r="AM6" s="7"/>
+      <x:c r="AN6" s="7"/>
+      <x:c r="AO6" s="7"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7"/>
@@ -688,6 +821,17 @@
       <x:c r="AB7" s="7"/>
       <x:c r="AC7" s="7"/>
       <x:c r="AD7" s="7"/>
+      <x:c r="AE7" s="7"/>
+      <x:c r="AF7" s="7"/>
+      <x:c r="AG7" s="7"/>
+      <x:c r="AH7" s="7"/>
+      <x:c r="AI7" s="7"/>
+      <x:c r="AJ7" s="7"/>
+      <x:c r="AK7" s="7"/>
+      <x:c r="AL7" s="7"/>
+      <x:c r="AM7" s="7"/>
+      <x:c r="AN7" s="7"/>
+      <x:c r="AO7" s="7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7"/>
@@ -720,6 +864,17 @@
       <x:c r="AB8" s="7"/>
       <x:c r="AC8" s="7"/>
       <x:c r="AD8" s="7"/>
+      <x:c r="AE8" s="7"/>
+      <x:c r="AF8" s="7"/>
+      <x:c r="AG8" s="7"/>
+      <x:c r="AH8" s="7"/>
+      <x:c r="AI8" s="7"/>
+      <x:c r="AJ8" s="7"/>
+      <x:c r="AK8" s="7"/>
+      <x:c r="AL8" s="7"/>
+      <x:c r="AM8" s="7"/>
+      <x:c r="AN8" s="7"/>
+      <x:c r="AO8" s="7"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7"/>
@@ -752,6 +907,17 @@
       <x:c r="AB9" s="7"/>
       <x:c r="AC9" s="7"/>
       <x:c r="AD9" s="7"/>
+      <x:c r="AE9" s="7"/>
+      <x:c r="AF9" s="7"/>
+      <x:c r="AG9" s="7"/>
+      <x:c r="AH9" s="7"/>
+      <x:c r="AI9" s="7"/>
+      <x:c r="AJ9" s="7"/>
+      <x:c r="AK9" s="7"/>
+      <x:c r="AL9" s="7"/>
+      <x:c r="AM9" s="7"/>
+      <x:c r="AN9" s="7"/>
+      <x:c r="AO9" s="7"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7"/>
@@ -784,6 +950,17 @@
       <x:c r="AB10" s="7"/>
       <x:c r="AC10" s="7"/>
       <x:c r="AD10" s="7"/>
+      <x:c r="AE10" s="7"/>
+      <x:c r="AF10" s="7"/>
+      <x:c r="AG10" s="7"/>
+      <x:c r="AH10" s="7"/>
+      <x:c r="AI10" s="7"/>
+      <x:c r="AJ10" s="7"/>
+      <x:c r="AK10" s="7"/>
+      <x:c r="AL10" s="7"/>
+      <x:c r="AM10" s="7"/>
+      <x:c r="AN10" s="7"/>
+      <x:c r="AO10" s="7"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7"/>
@@ -816,6 +993,17 @@
       <x:c r="AB11" s="7"/>
       <x:c r="AC11" s="7"/>
       <x:c r="AD11" s="7"/>
+      <x:c r="AE11" s="7"/>
+      <x:c r="AF11" s="7"/>
+      <x:c r="AG11" s="7"/>
+      <x:c r="AH11" s="7"/>
+      <x:c r="AI11" s="7"/>
+      <x:c r="AJ11" s="7"/>
+      <x:c r="AK11" s="7"/>
+      <x:c r="AL11" s="7"/>
+      <x:c r="AM11" s="7"/>
+      <x:c r="AN11" s="7"/>
+      <x:c r="AO11" s="7"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7"/>
@@ -848,6 +1036,17 @@
       <x:c r="AB12" s="7"/>
       <x:c r="AC12" s="7"/>
       <x:c r="AD12" s="7"/>
+      <x:c r="AE12" s="7"/>
+      <x:c r="AF12" s="7"/>
+      <x:c r="AG12" s="7"/>
+      <x:c r="AH12" s="7"/>
+      <x:c r="AI12" s="7"/>
+      <x:c r="AJ12" s="7"/>
+      <x:c r="AK12" s="7"/>
+      <x:c r="AL12" s="7"/>
+      <x:c r="AM12" s="7"/>
+      <x:c r="AN12" s="7"/>
+      <x:c r="AO12" s="7"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7"/>
@@ -880,6 +1079,17 @@
       <x:c r="AB13" s="7"/>
       <x:c r="AC13" s="7"/>
       <x:c r="AD13" s="7"/>
+      <x:c r="AE13" s="7"/>
+      <x:c r="AF13" s="7"/>
+      <x:c r="AG13" s="7"/>
+      <x:c r="AH13" s="7"/>
+      <x:c r="AI13" s="7"/>
+      <x:c r="AJ13" s="7"/>
+      <x:c r="AK13" s="7"/>
+      <x:c r="AL13" s="7"/>
+      <x:c r="AM13" s="7"/>
+      <x:c r="AN13" s="7"/>
+      <x:c r="AO13" s="7"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7"/>
@@ -912,6 +1122,17 @@
       <x:c r="AB14" s="7"/>
       <x:c r="AC14" s="7"/>
       <x:c r="AD14" s="7"/>
+      <x:c r="AE14" s="7"/>
+      <x:c r="AF14" s="7"/>
+      <x:c r="AG14" s="7"/>
+      <x:c r="AH14" s="7"/>
+      <x:c r="AI14" s="7"/>
+      <x:c r="AJ14" s="7"/>
+      <x:c r="AK14" s="7"/>
+      <x:c r="AL14" s="7"/>
+      <x:c r="AM14" s="7"/>
+      <x:c r="AN14" s="7"/>
+      <x:c r="AO14" s="7"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7"/>
@@ -944,6 +1165,17 @@
       <x:c r="AB15" s="7"/>
       <x:c r="AC15" s="7"/>
       <x:c r="AD15" s="7"/>
+      <x:c r="AE15" s="7"/>
+      <x:c r="AF15" s="7"/>
+      <x:c r="AG15" s="7"/>
+      <x:c r="AH15" s="7"/>
+      <x:c r="AI15" s="7"/>
+      <x:c r="AJ15" s="7"/>
+      <x:c r="AK15" s="7"/>
+      <x:c r="AL15" s="7"/>
+      <x:c r="AM15" s="7"/>
+      <x:c r="AN15" s="7"/>
+      <x:c r="AO15" s="7"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7"/>
@@ -976,6 +1208,17 @@
       <x:c r="AB16" s="7"/>
       <x:c r="AC16" s="7"/>
       <x:c r="AD16" s="7"/>
+      <x:c r="AE16" s="7"/>
+      <x:c r="AF16" s="7"/>
+      <x:c r="AG16" s="7"/>
+      <x:c r="AH16" s="7"/>
+      <x:c r="AI16" s="7"/>
+      <x:c r="AJ16" s="7"/>
+      <x:c r="AK16" s="7"/>
+      <x:c r="AL16" s="7"/>
+      <x:c r="AM16" s="7"/>
+      <x:c r="AN16" s="7"/>
+      <x:c r="AO16" s="7"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7"/>
@@ -1008,6 +1251,17 @@
       <x:c r="AB17" s="7"/>
       <x:c r="AC17" s="7"/>
       <x:c r="AD17" s="7"/>
+      <x:c r="AE17" s="7"/>
+      <x:c r="AF17" s="7"/>
+      <x:c r="AG17" s="7"/>
+      <x:c r="AH17" s="7"/>
+      <x:c r="AI17" s="7"/>
+      <x:c r="AJ17" s="7"/>
+      <x:c r="AK17" s="7"/>
+      <x:c r="AL17" s="7"/>
+      <x:c r="AM17" s="7"/>
+      <x:c r="AN17" s="7"/>
+      <x:c r="AO17" s="7"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7"/>
@@ -1040,6 +1294,17 @@
       <x:c r="AB18" s="7"/>
       <x:c r="AC18" s="7"/>
       <x:c r="AD18" s="7"/>
+      <x:c r="AE18" s="7"/>
+      <x:c r="AF18" s="7"/>
+      <x:c r="AG18" s="7"/>
+      <x:c r="AH18" s="7"/>
+      <x:c r="AI18" s="7"/>
+      <x:c r="AJ18" s="7"/>
+      <x:c r="AK18" s="7"/>
+      <x:c r="AL18" s="7"/>
+      <x:c r="AM18" s="7"/>
+      <x:c r="AN18" s="7"/>
+      <x:c r="AO18" s="7"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7"/>
@@ -1072,6 +1337,17 @@
       <x:c r="AB19" s="7"/>
       <x:c r="AC19" s="7"/>
       <x:c r="AD19" s="7"/>
+      <x:c r="AE19" s="7"/>
+      <x:c r="AF19" s="7"/>
+      <x:c r="AG19" s="7"/>
+      <x:c r="AH19" s="7"/>
+      <x:c r="AI19" s="7"/>
+      <x:c r="AJ19" s="7"/>
+      <x:c r="AK19" s="7"/>
+      <x:c r="AL19" s="7"/>
+      <x:c r="AM19" s="7"/>
+      <x:c r="AN19" s="7"/>
+      <x:c r="AO19" s="7"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7"/>
@@ -1104,6 +1380,17 @@
       <x:c r="AB20" s="7"/>
       <x:c r="AC20" s="7"/>
       <x:c r="AD20" s="7"/>
+      <x:c r="AE20" s="7"/>
+      <x:c r="AF20" s="7"/>
+      <x:c r="AG20" s="7"/>
+      <x:c r="AH20" s="7"/>
+      <x:c r="AI20" s="7"/>
+      <x:c r="AJ20" s="7"/>
+      <x:c r="AK20" s="7"/>
+      <x:c r="AL20" s="7"/>
+      <x:c r="AM20" s="7"/>
+      <x:c r="AN20" s="7"/>
+      <x:c r="AO20" s="7"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7"/>
@@ -1136,6 +1423,17 @@
       <x:c r="AB21" s="7"/>
       <x:c r="AC21" s="7"/>
       <x:c r="AD21" s="7"/>
+      <x:c r="AE21" s="7"/>
+      <x:c r="AF21" s="7"/>
+      <x:c r="AG21" s="7"/>
+      <x:c r="AH21" s="7"/>
+      <x:c r="AI21" s="7"/>
+      <x:c r="AJ21" s="7"/>
+      <x:c r="AK21" s="7"/>
+      <x:c r="AL21" s="7"/>
+      <x:c r="AM21" s="7"/>
+      <x:c r="AN21" s="7"/>
+      <x:c r="AO21" s="7"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="7"/>
@@ -1168,6 +1466,17 @@
       <x:c r="AB22" s="7"/>
       <x:c r="AC22" s="7"/>
       <x:c r="AD22" s="7"/>
+      <x:c r="AE22" s="7"/>
+      <x:c r="AF22" s="7"/>
+      <x:c r="AG22" s="7"/>
+      <x:c r="AH22" s="7"/>
+      <x:c r="AI22" s="7"/>
+      <x:c r="AJ22" s="7"/>
+      <x:c r="AK22" s="7"/>
+      <x:c r="AL22" s="7"/>
+      <x:c r="AM22" s="7"/>
+      <x:c r="AN22" s="7"/>
+      <x:c r="AO22" s="7"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7"/>
@@ -1200,6 +1509,17 @@
       <x:c r="AB23" s="7"/>
       <x:c r="AC23" s="7"/>
       <x:c r="AD23" s="7"/>
+      <x:c r="AE23" s="7"/>
+      <x:c r="AF23" s="7"/>
+      <x:c r="AG23" s="7"/>
+      <x:c r="AH23" s="7"/>
+      <x:c r="AI23" s="7"/>
+      <x:c r="AJ23" s="7"/>
+      <x:c r="AK23" s="7"/>
+      <x:c r="AL23" s="7"/>
+      <x:c r="AM23" s="7"/>
+      <x:c r="AN23" s="7"/>
+      <x:c r="AO23" s="7"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7"/>
@@ -1232,6 +1552,17 @@
       <x:c r="AB24" s="7"/>
       <x:c r="AC24" s="7"/>
       <x:c r="AD24" s="7"/>
+      <x:c r="AE24" s="7"/>
+      <x:c r="AF24" s="7"/>
+      <x:c r="AG24" s="7"/>
+      <x:c r="AH24" s="7"/>
+      <x:c r="AI24" s="7"/>
+      <x:c r="AJ24" s="7"/>
+      <x:c r="AK24" s="7"/>
+      <x:c r="AL24" s="7"/>
+      <x:c r="AM24" s="7"/>
+      <x:c r="AN24" s="7"/>
+      <x:c r="AO24" s="7"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="7"/>
@@ -1264,6 +1595,17 @@
       <x:c r="AB25" s="7"/>
       <x:c r="AC25" s="7"/>
       <x:c r="AD25" s="7"/>
+      <x:c r="AE25" s="7"/>
+      <x:c r="AF25" s="7"/>
+      <x:c r="AG25" s="7"/>
+      <x:c r="AH25" s="7"/>
+      <x:c r="AI25" s="7"/>
+      <x:c r="AJ25" s="7"/>
+      <x:c r="AK25" s="7"/>
+      <x:c r="AL25" s="7"/>
+      <x:c r="AM25" s="7"/>
+      <x:c r="AN25" s="7"/>
+      <x:c r="AO25" s="7"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="7"/>
@@ -1296,6 +1638,17 @@
       <x:c r="AB26" s="7"/>
       <x:c r="AC26" s="7"/>
       <x:c r="AD26" s="7"/>
+      <x:c r="AE26" s="7"/>
+      <x:c r="AF26" s="7"/>
+      <x:c r="AG26" s="7"/>
+      <x:c r="AH26" s="7"/>
+      <x:c r="AI26" s="7"/>
+      <x:c r="AJ26" s="7"/>
+      <x:c r="AK26" s="7"/>
+      <x:c r="AL26" s="7"/>
+      <x:c r="AM26" s="7"/>
+      <x:c r="AN26" s="7"/>
+      <x:c r="AO26" s="7"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="7"/>
@@ -1328,6 +1681,17 @@
       <x:c r="AB27" s="7"/>
       <x:c r="AC27" s="7"/>
       <x:c r="AD27" s="7"/>
+      <x:c r="AE27" s="7"/>
+      <x:c r="AF27" s="7"/>
+      <x:c r="AG27" s="7"/>
+      <x:c r="AH27" s="7"/>
+      <x:c r="AI27" s="7"/>
+      <x:c r="AJ27" s="7"/>
+      <x:c r="AK27" s="7"/>
+      <x:c r="AL27" s="7"/>
+      <x:c r="AM27" s="7"/>
+      <x:c r="AN27" s="7"/>
+      <x:c r="AO27" s="7"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="7"/>
@@ -1360,6 +1724,17 @@
       <x:c r="AB28" s="7"/>
       <x:c r="AC28" s="7"/>
       <x:c r="AD28" s="7"/>
+      <x:c r="AE28" s="7"/>
+      <x:c r="AF28" s="7"/>
+      <x:c r="AG28" s="7"/>
+      <x:c r="AH28" s="7"/>
+      <x:c r="AI28" s="7"/>
+      <x:c r="AJ28" s="7"/>
+      <x:c r="AK28" s="7"/>
+      <x:c r="AL28" s="7"/>
+      <x:c r="AM28" s="7"/>
+      <x:c r="AN28" s="7"/>
+      <x:c r="AO28" s="7"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="7"/>
@@ -1392,6 +1767,17 @@
       <x:c r="AB29" s="7"/>
       <x:c r="AC29" s="7"/>
       <x:c r="AD29" s="7"/>
+      <x:c r="AE29" s="7"/>
+      <x:c r="AF29" s="7"/>
+      <x:c r="AG29" s="7"/>
+      <x:c r="AH29" s="7"/>
+      <x:c r="AI29" s="7"/>
+      <x:c r="AJ29" s="7"/>
+      <x:c r="AK29" s="7"/>
+      <x:c r="AL29" s="7"/>
+      <x:c r="AM29" s="7"/>
+      <x:c r="AN29" s="7"/>
+      <x:c r="AO29" s="7"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="7"/>
@@ -1424,6 +1810,17 @@
       <x:c r="AB30" s="7"/>
       <x:c r="AC30" s="7"/>
       <x:c r="AD30" s="7"/>
+      <x:c r="AE30" s="7"/>
+      <x:c r="AF30" s="7"/>
+      <x:c r="AG30" s="7"/>
+      <x:c r="AH30" s="7"/>
+      <x:c r="AI30" s="7"/>
+      <x:c r="AJ30" s="7"/>
+      <x:c r="AK30" s="7"/>
+      <x:c r="AL30" s="7"/>
+      <x:c r="AM30" s="7"/>
+      <x:c r="AN30" s="7"/>
+      <x:c r="AO30" s="7"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="7"/>
@@ -1456,6 +1853,17 @@
       <x:c r="AB31" s="7"/>
       <x:c r="AC31" s="7"/>
       <x:c r="AD31" s="7"/>
+      <x:c r="AE31" s="7"/>
+      <x:c r="AF31" s="7"/>
+      <x:c r="AG31" s="7"/>
+      <x:c r="AH31" s="7"/>
+      <x:c r="AI31" s="7"/>
+      <x:c r="AJ31" s="7"/>
+      <x:c r="AK31" s="7"/>
+      <x:c r="AL31" s="7"/>
+      <x:c r="AM31" s="7"/>
+      <x:c r="AN31" s="7"/>
+      <x:c r="AO31" s="7"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="7"/>
@@ -1488,6 +1896,17 @@
       <x:c r="AB32" s="7"/>
       <x:c r="AC32" s="7"/>
       <x:c r="AD32" s="7"/>
+      <x:c r="AE32" s="7"/>
+      <x:c r="AF32" s="7"/>
+      <x:c r="AG32" s="7"/>
+      <x:c r="AH32" s="7"/>
+      <x:c r="AI32" s="7"/>
+      <x:c r="AJ32" s="7"/>
+      <x:c r="AK32" s="7"/>
+      <x:c r="AL32" s="7"/>
+      <x:c r="AM32" s="7"/>
+      <x:c r="AN32" s="7"/>
+      <x:c r="AO32" s="7"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="7"/>
@@ -1520,6 +1939,17 @@
       <x:c r="AB33" s="7"/>
       <x:c r="AC33" s="7"/>
       <x:c r="AD33" s="7"/>
+      <x:c r="AE33" s="7"/>
+      <x:c r="AF33" s="7"/>
+      <x:c r="AG33" s="7"/>
+      <x:c r="AH33" s="7"/>
+      <x:c r="AI33" s="7"/>
+      <x:c r="AJ33" s="7"/>
+      <x:c r="AK33" s="7"/>
+      <x:c r="AL33" s="7"/>
+      <x:c r="AM33" s="7"/>
+      <x:c r="AN33" s="7"/>
+      <x:c r="AO33" s="7"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="7"/>
@@ -1552,6 +1982,17 @@
       <x:c r="AB34" s="7"/>
       <x:c r="AC34" s="7"/>
       <x:c r="AD34" s="7"/>
+      <x:c r="AE34" s="7"/>
+      <x:c r="AF34" s="7"/>
+      <x:c r="AG34" s="7"/>
+      <x:c r="AH34" s="7"/>
+      <x:c r="AI34" s="7"/>
+      <x:c r="AJ34" s="7"/>
+      <x:c r="AK34" s="7"/>
+      <x:c r="AL34" s="7"/>
+      <x:c r="AM34" s="7"/>
+      <x:c r="AN34" s="7"/>
+      <x:c r="AO34" s="7"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="7"/>
@@ -1584,6 +2025,17 @@
       <x:c r="AB35" s="7"/>
       <x:c r="AC35" s="7"/>
       <x:c r="AD35" s="7"/>
+      <x:c r="AE35" s="7"/>
+      <x:c r="AF35" s="7"/>
+      <x:c r="AG35" s="7"/>
+      <x:c r="AH35" s="7"/>
+      <x:c r="AI35" s="7"/>
+      <x:c r="AJ35" s="7"/>
+      <x:c r="AK35" s="7"/>
+      <x:c r="AL35" s="7"/>
+      <x:c r="AM35" s="7"/>
+      <x:c r="AN35" s="7"/>
+      <x:c r="AO35" s="7"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="7"/>
@@ -1616,6 +2068,17 @@
       <x:c r="AB36" s="7"/>
       <x:c r="AC36" s="7"/>
       <x:c r="AD36" s="7"/>
+      <x:c r="AE36" s="7"/>
+      <x:c r="AF36" s="7"/>
+      <x:c r="AG36" s="7"/>
+      <x:c r="AH36" s="7"/>
+      <x:c r="AI36" s="7"/>
+      <x:c r="AJ36" s="7"/>
+      <x:c r="AK36" s="7"/>
+      <x:c r="AL36" s="7"/>
+      <x:c r="AM36" s="7"/>
+      <x:c r="AN36" s="7"/>
+      <x:c r="AO36" s="7"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="7"/>
@@ -1648,6 +2111,17 @@
       <x:c r="AB37" s="7"/>
       <x:c r="AC37" s="7"/>
       <x:c r="AD37" s="7"/>
+      <x:c r="AE37" s="7"/>
+      <x:c r="AF37" s="7"/>
+      <x:c r="AG37" s="7"/>
+      <x:c r="AH37" s="7"/>
+      <x:c r="AI37" s="7"/>
+      <x:c r="AJ37" s="7"/>
+      <x:c r="AK37" s="7"/>
+      <x:c r="AL37" s="7"/>
+      <x:c r="AM37" s="7"/>
+      <x:c r="AN37" s="7"/>
+      <x:c r="AO37" s="7"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="7"/>
@@ -1680,6 +2154,17 @@
       <x:c r="AB38" s="7"/>
       <x:c r="AC38" s="7"/>
       <x:c r="AD38" s="7"/>
+      <x:c r="AE38" s="7"/>
+      <x:c r="AF38" s="7"/>
+      <x:c r="AG38" s="7"/>
+      <x:c r="AH38" s="7"/>
+      <x:c r="AI38" s="7"/>
+      <x:c r="AJ38" s="7"/>
+      <x:c r="AK38" s="7"/>
+      <x:c r="AL38" s="7"/>
+      <x:c r="AM38" s="7"/>
+      <x:c r="AN38" s="7"/>
+      <x:c r="AO38" s="7"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="7"/>
@@ -1712,6 +2197,17 @@
       <x:c r="AB39" s="7"/>
       <x:c r="AC39" s="7"/>
       <x:c r="AD39" s="7"/>
+      <x:c r="AE39" s="7"/>
+      <x:c r="AF39" s="7"/>
+      <x:c r="AG39" s="7"/>
+      <x:c r="AH39" s="7"/>
+      <x:c r="AI39" s="7"/>
+      <x:c r="AJ39" s="7"/>
+      <x:c r="AK39" s="7"/>
+      <x:c r="AL39" s="7"/>
+      <x:c r="AM39" s="7"/>
+      <x:c r="AN39" s="7"/>
+      <x:c r="AO39" s="7"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="7"/>
@@ -1744,6 +2240,17 @@
       <x:c r="AB40" s="7"/>
       <x:c r="AC40" s="7"/>
       <x:c r="AD40" s="7"/>
+      <x:c r="AE40" s="7"/>
+      <x:c r="AF40" s="7"/>
+      <x:c r="AG40" s="7"/>
+      <x:c r="AH40" s="7"/>
+      <x:c r="AI40" s="7"/>
+      <x:c r="AJ40" s="7"/>
+      <x:c r="AK40" s="7"/>
+      <x:c r="AL40" s="7"/>
+      <x:c r="AM40" s="7"/>
+      <x:c r="AN40" s="7"/>
+      <x:c r="AO40" s="7"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="7"/>
@@ -1776,6 +2283,17 @@
       <x:c r="AB41" s="7"/>
       <x:c r="AC41" s="7"/>
       <x:c r="AD41" s="7"/>
+      <x:c r="AE41" s="7"/>
+      <x:c r="AF41" s="7"/>
+      <x:c r="AG41" s="7"/>
+      <x:c r="AH41" s="7"/>
+      <x:c r="AI41" s="7"/>
+      <x:c r="AJ41" s="7"/>
+      <x:c r="AK41" s="7"/>
+      <x:c r="AL41" s="7"/>
+      <x:c r="AM41" s="7"/>
+      <x:c r="AN41" s="7"/>
+      <x:c r="AO41" s="7"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="7"/>
@@ -1808,6 +2326,17 @@
       <x:c r="AB42" s="7"/>
       <x:c r="AC42" s="7"/>
       <x:c r="AD42" s="7"/>
+      <x:c r="AE42" s="7"/>
+      <x:c r="AF42" s="7"/>
+      <x:c r="AG42" s="7"/>
+      <x:c r="AH42" s="7"/>
+      <x:c r="AI42" s="7"/>
+      <x:c r="AJ42" s="7"/>
+      <x:c r="AK42" s="7"/>
+      <x:c r="AL42" s="7"/>
+      <x:c r="AM42" s="7"/>
+      <x:c r="AN42" s="7"/>
+      <x:c r="AO42" s="7"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="7"/>
@@ -1840,6 +2369,17 @@
       <x:c r="AB43" s="7"/>
       <x:c r="AC43" s="7"/>
       <x:c r="AD43" s="7"/>
+      <x:c r="AE43" s="7"/>
+      <x:c r="AF43" s="7"/>
+      <x:c r="AG43" s="7"/>
+      <x:c r="AH43" s="7"/>
+      <x:c r="AI43" s="7"/>
+      <x:c r="AJ43" s="7"/>
+      <x:c r="AK43" s="7"/>
+      <x:c r="AL43" s="7"/>
+      <x:c r="AM43" s="7"/>
+      <x:c r="AN43" s="7"/>
+      <x:c r="AO43" s="7"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="7"/>
@@ -1872,6 +2412,17 @@
       <x:c r="AB44" s="7"/>
       <x:c r="AC44" s="7"/>
       <x:c r="AD44" s="7"/>
+      <x:c r="AE44" s="7"/>
+      <x:c r="AF44" s="7"/>
+      <x:c r="AG44" s="7"/>
+      <x:c r="AH44" s="7"/>
+      <x:c r="AI44" s="7"/>
+      <x:c r="AJ44" s="7"/>
+      <x:c r="AK44" s="7"/>
+      <x:c r="AL44" s="7"/>
+      <x:c r="AM44" s="7"/>
+      <x:c r="AN44" s="7"/>
+      <x:c r="AO44" s="7"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="7"/>
@@ -1904,6 +2455,17 @@
       <x:c r="AB45" s="7"/>
       <x:c r="AC45" s="7"/>
       <x:c r="AD45" s="7"/>
+      <x:c r="AE45" s="7"/>
+      <x:c r="AF45" s="7"/>
+      <x:c r="AG45" s="7"/>
+      <x:c r="AH45" s="7"/>
+      <x:c r="AI45" s="7"/>
+      <x:c r="AJ45" s="7"/>
+      <x:c r="AK45" s="7"/>
+      <x:c r="AL45" s="7"/>
+      <x:c r="AM45" s="7"/>
+      <x:c r="AN45" s="7"/>
+      <x:c r="AO45" s="7"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="7"/>
@@ -1936,6 +2498,17 @@
       <x:c r="AB46" s="7"/>
       <x:c r="AC46" s="7"/>
       <x:c r="AD46" s="7"/>
+      <x:c r="AE46" s="7"/>
+      <x:c r="AF46" s="7"/>
+      <x:c r="AG46" s="7"/>
+      <x:c r="AH46" s="7"/>
+      <x:c r="AI46" s="7"/>
+      <x:c r="AJ46" s="7"/>
+      <x:c r="AK46" s="7"/>
+      <x:c r="AL46" s="7"/>
+      <x:c r="AM46" s="7"/>
+      <x:c r="AN46" s="7"/>
+      <x:c r="AO46" s="7"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="7"/>
@@ -1968,6 +2541,17 @@
       <x:c r="AB47" s="7"/>
       <x:c r="AC47" s="7"/>
       <x:c r="AD47" s="7"/>
+      <x:c r="AE47" s="7"/>
+      <x:c r="AF47" s="7"/>
+      <x:c r="AG47" s="7"/>
+      <x:c r="AH47" s="7"/>
+      <x:c r="AI47" s="7"/>
+      <x:c r="AJ47" s="7"/>
+      <x:c r="AK47" s="7"/>
+      <x:c r="AL47" s="7"/>
+      <x:c r="AM47" s="7"/>
+      <x:c r="AN47" s="7"/>
+      <x:c r="AO47" s="7"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="7"/>
@@ -2000,6 +2584,17 @@
       <x:c r="AB48" s="7"/>
       <x:c r="AC48" s="7"/>
       <x:c r="AD48" s="7"/>
+      <x:c r="AE48" s="7"/>
+      <x:c r="AF48" s="7"/>
+      <x:c r="AG48" s="7"/>
+      <x:c r="AH48" s="7"/>
+      <x:c r="AI48" s="7"/>
+      <x:c r="AJ48" s="7"/>
+      <x:c r="AK48" s="7"/>
+      <x:c r="AL48" s="7"/>
+      <x:c r="AM48" s="7"/>
+      <x:c r="AN48" s="7"/>
+      <x:c r="AO48" s="7"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="7"/>
@@ -2032,6 +2627,17 @@
       <x:c r="AB49" s="7"/>
       <x:c r="AC49" s="7"/>
       <x:c r="AD49" s="7"/>
+      <x:c r="AE49" s="7"/>
+      <x:c r="AF49" s="7"/>
+      <x:c r="AG49" s="7"/>
+      <x:c r="AH49" s="7"/>
+      <x:c r="AI49" s="7"/>
+      <x:c r="AJ49" s="7"/>
+      <x:c r="AK49" s="7"/>
+      <x:c r="AL49" s="7"/>
+      <x:c r="AM49" s="7"/>
+      <x:c r="AN49" s="7"/>
+      <x:c r="AO49" s="7"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="7"/>
@@ -2064,6 +2670,17 @@
       <x:c r="AB50" s="7"/>
       <x:c r="AC50" s="7"/>
       <x:c r="AD50" s="7"/>
+      <x:c r="AE50" s="7"/>
+      <x:c r="AF50" s="7"/>
+      <x:c r="AG50" s="7"/>
+      <x:c r="AH50" s="7"/>
+      <x:c r="AI50" s="7"/>
+      <x:c r="AJ50" s="7"/>
+      <x:c r="AK50" s="7"/>
+      <x:c r="AL50" s="7"/>
+      <x:c r="AM50" s="7"/>
+      <x:c r="AN50" s="7"/>
+      <x:c r="AO50" s="7"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="7"/>
@@ -2096,6 +2713,17 @@
       <x:c r="AB51" s="7"/>
       <x:c r="AC51" s="7"/>
       <x:c r="AD51" s="7"/>
+      <x:c r="AE51" s="7"/>
+      <x:c r="AF51" s="7"/>
+      <x:c r="AG51" s="7"/>
+      <x:c r="AH51" s="7"/>
+      <x:c r="AI51" s="7"/>
+      <x:c r="AJ51" s="7"/>
+      <x:c r="AK51" s="7"/>
+      <x:c r="AL51" s="7"/>
+      <x:c r="AM51" s="7"/>
+      <x:c r="AN51" s="7"/>
+      <x:c r="AO51" s="7"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
@@ -2111,7 +2739,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R689600b279064faf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e34e75f29f74d7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2138,6 +2766,17 @@
     <x:col min="16" max="16" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="18.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2193,7 +2832,40 @@
         <x:v>Sub-pods</x:v>
       </x:c>
       <x:c r="R1" s="4" t="str">
-        <x:v>Campaign</x:v>
+        <x:v>Campaign 1</x:v>
+      </x:c>
+      <x:c r="S1" s="4" t="str">
+        <x:v>Campaign 1 Status</x:v>
+      </x:c>
+      <x:c r="T1" s="4" t="str">
+        <x:v>Campaign 1 Target Commitment</x:v>
+      </x:c>
+      <x:c r="U1" s="4" t="str">
+        <x:v>Campaign 2</x:v>
+      </x:c>
+      <x:c r="V1" s="4" t="str">
+        <x:v>Campaign 2 Status</x:v>
+      </x:c>
+      <x:c r="W1" s="4" t="str">
+        <x:v>Campaign 2 Target Commitment</x:v>
+      </x:c>
+      <x:c r="X1" s="4" t="str">
+        <x:v>Campaign 3</x:v>
+      </x:c>
+      <x:c r="Y1" s="4" t="str">
+        <x:v>Campaign 3 Status</x:v>
+      </x:c>
+      <x:c r="Z1" s="4" t="str">
+        <x:v>Campaign 3 Target Commitment</x:v>
+      </x:c>
+      <x:c r="AA1" s="4" t="str">
+        <x:v>Campaign 4</x:v>
+      </x:c>
+      <x:c r="AB1" s="4" t="str">
+        <x:v>Campaign 4 Status</x:v>
+      </x:c>
+      <x:c r="AC1" s="4" t="str">
+        <x:v>Campaign 4 Target Commitment</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -2248,7 +2920,24 @@
       <x:c r="Q2" s="7" t="str">
         <x:v>LP Internal</x:v>
       </x:c>
-      <x:c r="R2" s="7" t="str"/>
+      <x:c r="R2" s="7" t="str">
+        <x:v>Kinship Fund Pipeline</x:v>
+      </x:c>
+      <x:c r="S2" s="7" t="str">
+        <x:v>Closed/Won</x:v>
+      </x:c>
+      <x:c r="T2" s="7" t="str">
+        <x:v>500000</x:v>
+      </x:c>
+      <x:c r="U2" s="7" t="str"/>
+      <x:c r="V2" s="7" t="str"/>
+      <x:c r="W2" s="7" t="str"/>
+      <x:c r="X2" s="7" t="str"/>
+      <x:c r="Y2" s="7" t="str"/>
+      <x:c r="Z2" s="7" t="str"/>
+      <x:c r="AA2" s="7" t="str"/>
+      <x:c r="AB2" s="7" t="str"/>
+      <x:c r="AC2" s="7" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str"/>
@@ -2269,6 +2958,17 @@
       <x:c r="P3" s="7" t="str"/>
       <x:c r="Q3" s="7" t="str"/>
       <x:c r="R3" s="7" t="str"/>
+      <x:c r="S3" s="7" t="str"/>
+      <x:c r="T3" s="7" t="str"/>
+      <x:c r="U3" s="7" t="str"/>
+      <x:c r="V3" s="7" t="str"/>
+      <x:c r="W3" s="7" t="str"/>
+      <x:c r="X3" s="7" t="str"/>
+      <x:c r="Y3" s="7" t="str"/>
+      <x:c r="Z3" s="7" t="str"/>
+      <x:c r="AA3" s="7" t="str"/>
+      <x:c r="AB3" s="7" t="str"/>
+      <x:c r="AC3" s="7" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str"/>
@@ -2289,6 +2989,17 @@
       <x:c r="P4" s="7" t="str"/>
       <x:c r="Q4" s="7" t="str"/>
       <x:c r="R4" s="7" t="str"/>
+      <x:c r="S4" s="7" t="str"/>
+      <x:c r="T4" s="7" t="str"/>
+      <x:c r="U4" s="7" t="str"/>
+      <x:c r="V4" s="7" t="str"/>
+      <x:c r="W4" s="7" t="str"/>
+      <x:c r="X4" s="7" t="str"/>
+      <x:c r="Y4" s="7" t="str"/>
+      <x:c r="Z4" s="7" t="str"/>
+      <x:c r="AA4" s="7" t="str"/>
+      <x:c r="AB4" s="7" t="str"/>
+      <x:c r="AC4" s="7" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="7"/>
@@ -2309,6 +3020,17 @@
       <x:c r="P5" s="7"/>
       <x:c r="Q5" s="7"/>
       <x:c r="R5" s="7"/>
+      <x:c r="S5" s="7"/>
+      <x:c r="T5" s="7"/>
+      <x:c r="U5" s="7"/>
+      <x:c r="V5" s="7"/>
+      <x:c r="W5" s="7"/>
+      <x:c r="X5" s="7"/>
+      <x:c r="Y5" s="7"/>
+      <x:c r="Z5" s="7"/>
+      <x:c r="AA5" s="7"/>
+      <x:c r="AB5" s="7"/>
+      <x:c r="AC5" s="7"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7"/>
@@ -2329,6 +3051,17 @@
       <x:c r="P6" s="7"/>
       <x:c r="Q6" s="7"/>
       <x:c r="R6" s="7"/>
+      <x:c r="S6" s="7"/>
+      <x:c r="T6" s="7"/>
+      <x:c r="U6" s="7"/>
+      <x:c r="V6" s="7"/>
+      <x:c r="W6" s="7"/>
+      <x:c r="X6" s="7"/>
+      <x:c r="Y6" s="7"/>
+      <x:c r="Z6" s="7"/>
+      <x:c r="AA6" s="7"/>
+      <x:c r="AB6" s="7"/>
+      <x:c r="AC6" s="7"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7"/>
@@ -2349,6 +3082,17 @@
       <x:c r="P7" s="7"/>
       <x:c r="Q7" s="7"/>
       <x:c r="R7" s="7"/>
+      <x:c r="S7" s="7"/>
+      <x:c r="T7" s="7"/>
+      <x:c r="U7" s="7"/>
+      <x:c r="V7" s="7"/>
+      <x:c r="W7" s="7"/>
+      <x:c r="X7" s="7"/>
+      <x:c r="Y7" s="7"/>
+      <x:c r="Z7" s="7"/>
+      <x:c r="AA7" s="7"/>
+      <x:c r="AB7" s="7"/>
+      <x:c r="AC7" s="7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7"/>
@@ -2369,6 +3113,17 @@
       <x:c r="P8" s="7"/>
       <x:c r="Q8" s="7"/>
       <x:c r="R8" s="7"/>
+      <x:c r="S8" s="7"/>
+      <x:c r="T8" s="7"/>
+      <x:c r="U8" s="7"/>
+      <x:c r="V8" s="7"/>
+      <x:c r="W8" s="7"/>
+      <x:c r="X8" s="7"/>
+      <x:c r="Y8" s="7"/>
+      <x:c r="Z8" s="7"/>
+      <x:c r="AA8" s="7"/>
+      <x:c r="AB8" s="7"/>
+      <x:c r="AC8" s="7"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7"/>
@@ -2389,6 +3144,17 @@
       <x:c r="P9" s="7"/>
       <x:c r="Q9" s="7"/>
       <x:c r="R9" s="7"/>
+      <x:c r="S9" s="7"/>
+      <x:c r="T9" s="7"/>
+      <x:c r="U9" s="7"/>
+      <x:c r="V9" s="7"/>
+      <x:c r="W9" s="7"/>
+      <x:c r="X9" s="7"/>
+      <x:c r="Y9" s="7"/>
+      <x:c r="Z9" s="7"/>
+      <x:c r="AA9" s="7"/>
+      <x:c r="AB9" s="7"/>
+      <x:c r="AC9" s="7"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7"/>
@@ -2409,6 +3175,17 @@
       <x:c r="P10" s="7"/>
       <x:c r="Q10" s="7"/>
       <x:c r="R10" s="7"/>
+      <x:c r="S10" s="7"/>
+      <x:c r="T10" s="7"/>
+      <x:c r="U10" s="7"/>
+      <x:c r="V10" s="7"/>
+      <x:c r="W10" s="7"/>
+      <x:c r="X10" s="7"/>
+      <x:c r="Y10" s="7"/>
+      <x:c r="Z10" s="7"/>
+      <x:c r="AA10" s="7"/>
+      <x:c r="AB10" s="7"/>
+      <x:c r="AC10" s="7"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7"/>
@@ -2429,6 +3206,17 @@
       <x:c r="P11" s="7"/>
       <x:c r="Q11" s="7"/>
       <x:c r="R11" s="7"/>
+      <x:c r="S11" s="7"/>
+      <x:c r="T11" s="7"/>
+      <x:c r="U11" s="7"/>
+      <x:c r="V11" s="7"/>
+      <x:c r="W11" s="7"/>
+      <x:c r="X11" s="7"/>
+      <x:c r="Y11" s="7"/>
+      <x:c r="Z11" s="7"/>
+      <x:c r="AA11" s="7"/>
+      <x:c r="AB11" s="7"/>
+      <x:c r="AC11" s="7"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7"/>
@@ -2449,6 +3237,17 @@
       <x:c r="P12" s="7"/>
       <x:c r="Q12" s="7"/>
       <x:c r="R12" s="7"/>
+      <x:c r="S12" s="7"/>
+      <x:c r="T12" s="7"/>
+      <x:c r="U12" s="7"/>
+      <x:c r="V12" s="7"/>
+      <x:c r="W12" s="7"/>
+      <x:c r="X12" s="7"/>
+      <x:c r="Y12" s="7"/>
+      <x:c r="Z12" s="7"/>
+      <x:c r="AA12" s="7"/>
+      <x:c r="AB12" s="7"/>
+      <x:c r="AC12" s="7"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7"/>
@@ -2469,6 +3268,17 @@
       <x:c r="P13" s="7"/>
       <x:c r="Q13" s="7"/>
       <x:c r="R13" s="7"/>
+      <x:c r="S13" s="7"/>
+      <x:c r="T13" s="7"/>
+      <x:c r="U13" s="7"/>
+      <x:c r="V13" s="7"/>
+      <x:c r="W13" s="7"/>
+      <x:c r="X13" s="7"/>
+      <x:c r="Y13" s="7"/>
+      <x:c r="Z13" s="7"/>
+      <x:c r="AA13" s="7"/>
+      <x:c r="AB13" s="7"/>
+      <x:c r="AC13" s="7"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7"/>
@@ -2489,6 +3299,17 @@
       <x:c r="P14" s="7"/>
       <x:c r="Q14" s="7"/>
       <x:c r="R14" s="7"/>
+      <x:c r="S14" s="7"/>
+      <x:c r="T14" s="7"/>
+      <x:c r="U14" s="7"/>
+      <x:c r="V14" s="7"/>
+      <x:c r="W14" s="7"/>
+      <x:c r="X14" s="7"/>
+      <x:c r="Y14" s="7"/>
+      <x:c r="Z14" s="7"/>
+      <x:c r="AA14" s="7"/>
+      <x:c r="AB14" s="7"/>
+      <x:c r="AC14" s="7"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7"/>
@@ -2509,6 +3330,17 @@
       <x:c r="P15" s="7"/>
       <x:c r="Q15" s="7"/>
       <x:c r="R15" s="7"/>
+      <x:c r="S15" s="7"/>
+      <x:c r="T15" s="7"/>
+      <x:c r="U15" s="7"/>
+      <x:c r="V15" s="7"/>
+      <x:c r="W15" s="7"/>
+      <x:c r="X15" s="7"/>
+      <x:c r="Y15" s="7"/>
+      <x:c r="Z15" s="7"/>
+      <x:c r="AA15" s="7"/>
+      <x:c r="AB15" s="7"/>
+      <x:c r="AC15" s="7"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7"/>
@@ -2529,6 +3361,17 @@
       <x:c r="P16" s="7"/>
       <x:c r="Q16" s="7"/>
       <x:c r="R16" s="7"/>
+      <x:c r="S16" s="7"/>
+      <x:c r="T16" s="7"/>
+      <x:c r="U16" s="7"/>
+      <x:c r="V16" s="7"/>
+      <x:c r="W16" s="7"/>
+      <x:c r="X16" s="7"/>
+      <x:c r="Y16" s="7"/>
+      <x:c r="Z16" s="7"/>
+      <x:c r="AA16" s="7"/>
+      <x:c r="AB16" s="7"/>
+      <x:c r="AC16" s="7"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7"/>
@@ -2549,6 +3392,17 @@
       <x:c r="P17" s="7"/>
       <x:c r="Q17" s="7"/>
       <x:c r="R17" s="7"/>
+      <x:c r="S17" s="7"/>
+      <x:c r="T17" s="7"/>
+      <x:c r="U17" s="7"/>
+      <x:c r="V17" s="7"/>
+      <x:c r="W17" s="7"/>
+      <x:c r="X17" s="7"/>
+      <x:c r="Y17" s="7"/>
+      <x:c r="Z17" s="7"/>
+      <x:c r="AA17" s="7"/>
+      <x:c r="AB17" s="7"/>
+      <x:c r="AC17" s="7"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7"/>
@@ -2569,6 +3423,17 @@
       <x:c r="P18" s="7"/>
       <x:c r="Q18" s="7"/>
       <x:c r="R18" s="7"/>
+      <x:c r="S18" s="7"/>
+      <x:c r="T18" s="7"/>
+      <x:c r="U18" s="7"/>
+      <x:c r="V18" s="7"/>
+      <x:c r="W18" s="7"/>
+      <x:c r="X18" s="7"/>
+      <x:c r="Y18" s="7"/>
+      <x:c r="Z18" s="7"/>
+      <x:c r="AA18" s="7"/>
+      <x:c r="AB18" s="7"/>
+      <x:c r="AC18" s="7"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7"/>
@@ -2589,6 +3454,17 @@
       <x:c r="P19" s="7"/>
       <x:c r="Q19" s="7"/>
       <x:c r="R19" s="7"/>
+      <x:c r="S19" s="7"/>
+      <x:c r="T19" s="7"/>
+      <x:c r="U19" s="7"/>
+      <x:c r="V19" s="7"/>
+      <x:c r="W19" s="7"/>
+      <x:c r="X19" s="7"/>
+      <x:c r="Y19" s="7"/>
+      <x:c r="Z19" s="7"/>
+      <x:c r="AA19" s="7"/>
+      <x:c r="AB19" s="7"/>
+      <x:c r="AC19" s="7"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7"/>
@@ -2609,6 +3485,17 @@
       <x:c r="P20" s="7"/>
       <x:c r="Q20" s="7"/>
       <x:c r="R20" s="7"/>
+      <x:c r="S20" s="7"/>
+      <x:c r="T20" s="7"/>
+      <x:c r="U20" s="7"/>
+      <x:c r="V20" s="7"/>
+      <x:c r="W20" s="7"/>
+      <x:c r="X20" s="7"/>
+      <x:c r="Y20" s="7"/>
+      <x:c r="Z20" s="7"/>
+      <x:c r="AA20" s="7"/>
+      <x:c r="AB20" s="7"/>
+      <x:c r="AC20" s="7"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7"/>
@@ -2629,6 +3516,17 @@
       <x:c r="P21" s="7"/>
       <x:c r="Q21" s="7"/>
       <x:c r="R21" s="7"/>
+      <x:c r="S21" s="7"/>
+      <x:c r="T21" s="7"/>
+      <x:c r="U21" s="7"/>
+      <x:c r="V21" s="7"/>
+      <x:c r="W21" s="7"/>
+      <x:c r="X21" s="7"/>
+      <x:c r="Y21" s="7"/>
+      <x:c r="Z21" s="7"/>
+      <x:c r="AA21" s="7"/>
+      <x:c r="AB21" s="7"/>
+      <x:c r="AC21" s="7"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="7"/>
@@ -2649,6 +3547,17 @@
       <x:c r="P22" s="7"/>
       <x:c r="Q22" s="7"/>
       <x:c r="R22" s="7"/>
+      <x:c r="S22" s="7"/>
+      <x:c r="T22" s="7"/>
+      <x:c r="U22" s="7"/>
+      <x:c r="V22" s="7"/>
+      <x:c r="W22" s="7"/>
+      <x:c r="X22" s="7"/>
+      <x:c r="Y22" s="7"/>
+      <x:c r="Z22" s="7"/>
+      <x:c r="AA22" s="7"/>
+      <x:c r="AB22" s="7"/>
+      <x:c r="AC22" s="7"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7"/>
@@ -2669,6 +3578,17 @@
       <x:c r="P23" s="7"/>
       <x:c r="Q23" s="7"/>
       <x:c r="R23" s="7"/>
+      <x:c r="S23" s="7"/>
+      <x:c r="T23" s="7"/>
+      <x:c r="U23" s="7"/>
+      <x:c r="V23" s="7"/>
+      <x:c r="W23" s="7"/>
+      <x:c r="X23" s="7"/>
+      <x:c r="Y23" s="7"/>
+      <x:c r="Z23" s="7"/>
+      <x:c r="AA23" s="7"/>
+      <x:c r="AB23" s="7"/>
+      <x:c r="AC23" s="7"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7"/>
@@ -2689,6 +3609,17 @@
       <x:c r="P24" s="7"/>
       <x:c r="Q24" s="7"/>
       <x:c r="R24" s="7"/>
+      <x:c r="S24" s="7"/>
+      <x:c r="T24" s="7"/>
+      <x:c r="U24" s="7"/>
+      <x:c r="V24" s="7"/>
+      <x:c r="W24" s="7"/>
+      <x:c r="X24" s="7"/>
+      <x:c r="Y24" s="7"/>
+      <x:c r="Z24" s="7"/>
+      <x:c r="AA24" s="7"/>
+      <x:c r="AB24" s="7"/>
+      <x:c r="AC24" s="7"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="7"/>
@@ -2709,6 +3640,17 @@
       <x:c r="P25" s="7"/>
       <x:c r="Q25" s="7"/>
       <x:c r="R25" s="7"/>
+      <x:c r="S25" s="7"/>
+      <x:c r="T25" s="7"/>
+      <x:c r="U25" s="7"/>
+      <x:c r="V25" s="7"/>
+      <x:c r="W25" s="7"/>
+      <x:c r="X25" s="7"/>
+      <x:c r="Y25" s="7"/>
+      <x:c r="Z25" s="7"/>
+      <x:c r="AA25" s="7"/>
+      <x:c r="AB25" s="7"/>
+      <x:c r="AC25" s="7"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="7"/>
@@ -2729,6 +3671,17 @@
       <x:c r="P26" s="7"/>
       <x:c r="Q26" s="7"/>
       <x:c r="R26" s="7"/>
+      <x:c r="S26" s="7"/>
+      <x:c r="T26" s="7"/>
+      <x:c r="U26" s="7"/>
+      <x:c r="V26" s="7"/>
+      <x:c r="W26" s="7"/>
+      <x:c r="X26" s="7"/>
+      <x:c r="Y26" s="7"/>
+      <x:c r="Z26" s="7"/>
+      <x:c r="AA26" s="7"/>
+      <x:c r="AB26" s="7"/>
+      <x:c r="AC26" s="7"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="7"/>
@@ -2749,6 +3702,17 @@
       <x:c r="P27" s="7"/>
       <x:c r="Q27" s="7"/>
       <x:c r="R27" s="7"/>
+      <x:c r="S27" s="7"/>
+      <x:c r="T27" s="7"/>
+      <x:c r="U27" s="7"/>
+      <x:c r="V27" s="7"/>
+      <x:c r="W27" s="7"/>
+      <x:c r="X27" s="7"/>
+      <x:c r="Y27" s="7"/>
+      <x:c r="Z27" s="7"/>
+      <x:c r="AA27" s="7"/>
+      <x:c r="AB27" s="7"/>
+      <x:c r="AC27" s="7"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="7"/>
@@ -2769,6 +3733,17 @@
       <x:c r="P28" s="7"/>
       <x:c r="Q28" s="7"/>
       <x:c r="R28" s="7"/>
+      <x:c r="S28" s="7"/>
+      <x:c r="T28" s="7"/>
+      <x:c r="U28" s="7"/>
+      <x:c r="V28" s="7"/>
+      <x:c r="W28" s="7"/>
+      <x:c r="X28" s="7"/>
+      <x:c r="Y28" s="7"/>
+      <x:c r="Z28" s="7"/>
+      <x:c r="AA28" s="7"/>
+      <x:c r="AB28" s="7"/>
+      <x:c r="AC28" s="7"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="7"/>
@@ -2789,6 +3764,17 @@
       <x:c r="P29" s="7"/>
       <x:c r="Q29" s="7"/>
       <x:c r="R29" s="7"/>
+      <x:c r="S29" s="7"/>
+      <x:c r="T29" s="7"/>
+      <x:c r="U29" s="7"/>
+      <x:c r="V29" s="7"/>
+      <x:c r="W29" s="7"/>
+      <x:c r="X29" s="7"/>
+      <x:c r="Y29" s="7"/>
+      <x:c r="Z29" s="7"/>
+      <x:c r="AA29" s="7"/>
+      <x:c r="AB29" s="7"/>
+      <x:c r="AC29" s="7"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="7"/>
@@ -2809,6 +3795,17 @@
       <x:c r="P30" s="7"/>
       <x:c r="Q30" s="7"/>
       <x:c r="R30" s="7"/>
+      <x:c r="S30" s="7"/>
+      <x:c r="T30" s="7"/>
+      <x:c r="U30" s="7"/>
+      <x:c r="V30" s="7"/>
+      <x:c r="W30" s="7"/>
+      <x:c r="X30" s="7"/>
+      <x:c r="Y30" s="7"/>
+      <x:c r="Z30" s="7"/>
+      <x:c r="AA30" s="7"/>
+      <x:c r="AB30" s="7"/>
+      <x:c r="AC30" s="7"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="7"/>
@@ -2829,6 +3826,17 @@
       <x:c r="P31" s="7"/>
       <x:c r="Q31" s="7"/>
       <x:c r="R31" s="7"/>
+      <x:c r="S31" s="7"/>
+      <x:c r="T31" s="7"/>
+      <x:c r="U31" s="7"/>
+      <x:c r="V31" s="7"/>
+      <x:c r="W31" s="7"/>
+      <x:c r="X31" s="7"/>
+      <x:c r="Y31" s="7"/>
+      <x:c r="Z31" s="7"/>
+      <x:c r="AA31" s="7"/>
+      <x:c r="AB31" s="7"/>
+      <x:c r="AC31" s="7"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="7"/>
@@ -2849,6 +3857,17 @@
       <x:c r="P32" s="7"/>
       <x:c r="Q32" s="7"/>
       <x:c r="R32" s="7"/>
+      <x:c r="S32" s="7"/>
+      <x:c r="T32" s="7"/>
+      <x:c r="U32" s="7"/>
+      <x:c r="V32" s="7"/>
+      <x:c r="W32" s="7"/>
+      <x:c r="X32" s="7"/>
+      <x:c r="Y32" s="7"/>
+      <x:c r="Z32" s="7"/>
+      <x:c r="AA32" s="7"/>
+      <x:c r="AB32" s="7"/>
+      <x:c r="AC32" s="7"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="7"/>
@@ -2869,6 +3888,17 @@
       <x:c r="P33" s="7"/>
       <x:c r="Q33" s="7"/>
       <x:c r="R33" s="7"/>
+      <x:c r="S33" s="7"/>
+      <x:c r="T33" s="7"/>
+      <x:c r="U33" s="7"/>
+      <x:c r="V33" s="7"/>
+      <x:c r="W33" s="7"/>
+      <x:c r="X33" s="7"/>
+      <x:c r="Y33" s="7"/>
+      <x:c r="Z33" s="7"/>
+      <x:c r="AA33" s="7"/>
+      <x:c r="AB33" s="7"/>
+      <x:c r="AC33" s="7"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="7"/>
@@ -2889,6 +3919,17 @@
       <x:c r="P34" s="7"/>
       <x:c r="Q34" s="7"/>
       <x:c r="R34" s="7"/>
+      <x:c r="S34" s="7"/>
+      <x:c r="T34" s="7"/>
+      <x:c r="U34" s="7"/>
+      <x:c r="V34" s="7"/>
+      <x:c r="W34" s="7"/>
+      <x:c r="X34" s="7"/>
+      <x:c r="Y34" s="7"/>
+      <x:c r="Z34" s="7"/>
+      <x:c r="AA34" s="7"/>
+      <x:c r="AB34" s="7"/>
+      <x:c r="AC34" s="7"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="7"/>
@@ -2909,6 +3950,17 @@
       <x:c r="P35" s="7"/>
       <x:c r="Q35" s="7"/>
       <x:c r="R35" s="7"/>
+      <x:c r="S35" s="7"/>
+      <x:c r="T35" s="7"/>
+      <x:c r="U35" s="7"/>
+      <x:c r="V35" s="7"/>
+      <x:c r="W35" s="7"/>
+      <x:c r="X35" s="7"/>
+      <x:c r="Y35" s="7"/>
+      <x:c r="Z35" s="7"/>
+      <x:c r="AA35" s="7"/>
+      <x:c r="AB35" s="7"/>
+      <x:c r="AC35" s="7"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="7"/>
@@ -2929,6 +3981,17 @@
       <x:c r="P36" s="7"/>
       <x:c r="Q36" s="7"/>
       <x:c r="R36" s="7"/>
+      <x:c r="S36" s="7"/>
+      <x:c r="T36" s="7"/>
+      <x:c r="U36" s="7"/>
+      <x:c r="V36" s="7"/>
+      <x:c r="W36" s="7"/>
+      <x:c r="X36" s="7"/>
+      <x:c r="Y36" s="7"/>
+      <x:c r="Z36" s="7"/>
+      <x:c r="AA36" s="7"/>
+      <x:c r="AB36" s="7"/>
+      <x:c r="AC36" s="7"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="7"/>
@@ -2949,6 +4012,17 @@
       <x:c r="P37" s="7"/>
       <x:c r="Q37" s="7"/>
       <x:c r="R37" s="7"/>
+      <x:c r="S37" s="7"/>
+      <x:c r="T37" s="7"/>
+      <x:c r="U37" s="7"/>
+      <x:c r="V37" s="7"/>
+      <x:c r="W37" s="7"/>
+      <x:c r="X37" s="7"/>
+      <x:c r="Y37" s="7"/>
+      <x:c r="Z37" s="7"/>
+      <x:c r="AA37" s="7"/>
+      <x:c r="AB37" s="7"/>
+      <x:c r="AC37" s="7"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="7"/>
@@ -2969,6 +4043,17 @@
       <x:c r="P38" s="7"/>
       <x:c r="Q38" s="7"/>
       <x:c r="R38" s="7"/>
+      <x:c r="S38" s="7"/>
+      <x:c r="T38" s="7"/>
+      <x:c r="U38" s="7"/>
+      <x:c r="V38" s="7"/>
+      <x:c r="W38" s="7"/>
+      <x:c r="X38" s="7"/>
+      <x:c r="Y38" s="7"/>
+      <x:c r="Z38" s="7"/>
+      <x:c r="AA38" s="7"/>
+      <x:c r="AB38" s="7"/>
+      <x:c r="AC38" s="7"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="7"/>
@@ -2989,6 +4074,17 @@
       <x:c r="P39" s="7"/>
       <x:c r="Q39" s="7"/>
       <x:c r="R39" s="7"/>
+      <x:c r="S39" s="7"/>
+      <x:c r="T39" s="7"/>
+      <x:c r="U39" s="7"/>
+      <x:c r="V39" s="7"/>
+      <x:c r="W39" s="7"/>
+      <x:c r="X39" s="7"/>
+      <x:c r="Y39" s="7"/>
+      <x:c r="Z39" s="7"/>
+      <x:c r="AA39" s="7"/>
+      <x:c r="AB39" s="7"/>
+      <x:c r="AC39" s="7"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="7"/>
@@ -3009,6 +4105,17 @@
       <x:c r="P40" s="7"/>
       <x:c r="Q40" s="7"/>
       <x:c r="R40" s="7"/>
+      <x:c r="S40" s="7"/>
+      <x:c r="T40" s="7"/>
+      <x:c r="U40" s="7"/>
+      <x:c r="V40" s="7"/>
+      <x:c r="W40" s="7"/>
+      <x:c r="X40" s="7"/>
+      <x:c r="Y40" s="7"/>
+      <x:c r="Z40" s="7"/>
+      <x:c r="AA40" s="7"/>
+      <x:c r="AB40" s="7"/>
+      <x:c r="AC40" s="7"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="7"/>
@@ -3029,6 +4136,17 @@
       <x:c r="P41" s="7"/>
       <x:c r="Q41" s="7"/>
       <x:c r="R41" s="7"/>
+      <x:c r="S41" s="7"/>
+      <x:c r="T41" s="7"/>
+      <x:c r="U41" s="7"/>
+      <x:c r="V41" s="7"/>
+      <x:c r="W41" s="7"/>
+      <x:c r="X41" s="7"/>
+      <x:c r="Y41" s="7"/>
+      <x:c r="Z41" s="7"/>
+      <x:c r="AA41" s="7"/>
+      <x:c r="AB41" s="7"/>
+      <x:c r="AC41" s="7"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="7"/>
@@ -3049,6 +4167,17 @@
       <x:c r="P42" s="7"/>
       <x:c r="Q42" s="7"/>
       <x:c r="R42" s="7"/>
+      <x:c r="S42" s="7"/>
+      <x:c r="T42" s="7"/>
+      <x:c r="U42" s="7"/>
+      <x:c r="V42" s="7"/>
+      <x:c r="W42" s="7"/>
+      <x:c r="X42" s="7"/>
+      <x:c r="Y42" s="7"/>
+      <x:c r="Z42" s="7"/>
+      <x:c r="AA42" s="7"/>
+      <x:c r="AB42" s="7"/>
+      <x:c r="AC42" s="7"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="7"/>
@@ -3069,6 +4198,17 @@
       <x:c r="P43" s="7"/>
       <x:c r="Q43" s="7"/>
       <x:c r="R43" s="7"/>
+      <x:c r="S43" s="7"/>
+      <x:c r="T43" s="7"/>
+      <x:c r="U43" s="7"/>
+      <x:c r="V43" s="7"/>
+      <x:c r="W43" s="7"/>
+      <x:c r="X43" s="7"/>
+      <x:c r="Y43" s="7"/>
+      <x:c r="Z43" s="7"/>
+      <x:c r="AA43" s="7"/>
+      <x:c r="AB43" s="7"/>
+      <x:c r="AC43" s="7"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="7"/>
@@ -3089,6 +4229,17 @@
       <x:c r="P44" s="7"/>
       <x:c r="Q44" s="7"/>
       <x:c r="R44" s="7"/>
+      <x:c r="S44" s="7"/>
+      <x:c r="T44" s="7"/>
+      <x:c r="U44" s="7"/>
+      <x:c r="V44" s="7"/>
+      <x:c r="W44" s="7"/>
+      <x:c r="X44" s="7"/>
+      <x:c r="Y44" s="7"/>
+      <x:c r="Z44" s="7"/>
+      <x:c r="AA44" s="7"/>
+      <x:c r="AB44" s="7"/>
+      <x:c r="AC44" s="7"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="7"/>
@@ -3109,6 +4260,17 @@
       <x:c r="P45" s="7"/>
       <x:c r="Q45" s="7"/>
       <x:c r="R45" s="7"/>
+      <x:c r="S45" s="7"/>
+      <x:c r="T45" s="7"/>
+      <x:c r="U45" s="7"/>
+      <x:c r="V45" s="7"/>
+      <x:c r="W45" s="7"/>
+      <x:c r="X45" s="7"/>
+      <x:c r="Y45" s="7"/>
+      <x:c r="Z45" s="7"/>
+      <x:c r="AA45" s="7"/>
+      <x:c r="AB45" s="7"/>
+      <x:c r="AC45" s="7"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="7"/>
@@ -3129,6 +4291,17 @@
       <x:c r="P46" s="7"/>
       <x:c r="Q46" s="7"/>
       <x:c r="R46" s="7"/>
+      <x:c r="S46" s="7"/>
+      <x:c r="T46" s="7"/>
+      <x:c r="U46" s="7"/>
+      <x:c r="V46" s="7"/>
+      <x:c r="W46" s="7"/>
+      <x:c r="X46" s="7"/>
+      <x:c r="Y46" s="7"/>
+      <x:c r="Z46" s="7"/>
+      <x:c r="AA46" s="7"/>
+      <x:c r="AB46" s="7"/>
+      <x:c r="AC46" s="7"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="7"/>
@@ -3149,6 +4322,17 @@
       <x:c r="P47" s="7"/>
       <x:c r="Q47" s="7"/>
       <x:c r="R47" s="7"/>
+      <x:c r="S47" s="7"/>
+      <x:c r="T47" s="7"/>
+      <x:c r="U47" s="7"/>
+      <x:c r="V47" s="7"/>
+      <x:c r="W47" s="7"/>
+      <x:c r="X47" s="7"/>
+      <x:c r="Y47" s="7"/>
+      <x:c r="Z47" s="7"/>
+      <x:c r="AA47" s="7"/>
+      <x:c r="AB47" s="7"/>
+      <x:c r="AC47" s="7"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="7"/>
@@ -3169,6 +4353,17 @@
       <x:c r="P48" s="7"/>
       <x:c r="Q48" s="7"/>
       <x:c r="R48" s="7"/>
+      <x:c r="S48" s="7"/>
+      <x:c r="T48" s="7"/>
+      <x:c r="U48" s="7"/>
+      <x:c r="V48" s="7"/>
+      <x:c r="W48" s="7"/>
+      <x:c r="X48" s="7"/>
+      <x:c r="Y48" s="7"/>
+      <x:c r="Z48" s="7"/>
+      <x:c r="AA48" s="7"/>
+      <x:c r="AB48" s="7"/>
+      <x:c r="AC48" s="7"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="7"/>
@@ -3189,6 +4384,17 @@
       <x:c r="P49" s="7"/>
       <x:c r="Q49" s="7"/>
       <x:c r="R49" s="7"/>
+      <x:c r="S49" s="7"/>
+      <x:c r="T49" s="7"/>
+      <x:c r="U49" s="7"/>
+      <x:c r="V49" s="7"/>
+      <x:c r="W49" s="7"/>
+      <x:c r="X49" s="7"/>
+      <x:c r="Y49" s="7"/>
+      <x:c r="Z49" s="7"/>
+      <x:c r="AA49" s="7"/>
+      <x:c r="AB49" s="7"/>
+      <x:c r="AC49" s="7"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="7"/>
@@ -3209,6 +4415,17 @@
       <x:c r="P50" s="7"/>
       <x:c r="Q50" s="7"/>
       <x:c r="R50" s="7"/>
+      <x:c r="S50" s="7"/>
+      <x:c r="T50" s="7"/>
+      <x:c r="U50" s="7"/>
+      <x:c r="V50" s="7"/>
+      <x:c r="W50" s="7"/>
+      <x:c r="X50" s="7"/>
+      <x:c r="Y50" s="7"/>
+      <x:c r="Z50" s="7"/>
+      <x:c r="AA50" s="7"/>
+      <x:c r="AB50" s="7"/>
+      <x:c r="AC50" s="7"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="7"/>
@@ -3229,6 +4446,17 @@
       <x:c r="P51" s="7"/>
       <x:c r="Q51" s="7"/>
       <x:c r="R51" s="7"/>
+      <x:c r="S51" s="7"/>
+      <x:c r="T51" s="7"/>
+      <x:c r="U51" s="7"/>
+      <x:c r="V51" s="7"/>
+      <x:c r="W51" s="7"/>
+      <x:c r="X51" s="7"/>
+      <x:c r="Y51" s="7"/>
+      <x:c r="Z51" s="7"/>
+      <x:c r="AA51" s="7"/>
+      <x:c r="AB51" s="7"/>
+      <x:c r="AC51" s="7"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -3238,7 +4466,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07c7e213345c476d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55f6de60a4d743d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>